<commit_message>
Planilhas: aplicar a rodada 7 da auditoria (metas: sentido obrigatório e média sem medição)
Dois achados nas três planilhas de metas (06 Completo, 19 Advogados, 19 Médicos),
reproduzidos antes de corrigir.

- R7-G1: o sentido entrou na guarda de entrada; vazio ou texto fora da lista deixa
  H vazio e J "Faltam dados" (antes caía no ramo "Maior é melhor" e um custo acima
  do teto virava "Atingido").
- R7-G2: média global e por objetivo testam COUNT(H) antes de calcular; sem nenhum
  progresso numérico escrevem "Faltam dados" (era 0 % via IFERROR, ou #DIV/0! por
  objetivo); a barra só desenha com número.
- Nota da aba atualizada; verificador do Completo com a mesma guarda.

Travas: recalc_todos 189.771 fórmulas / 0 erro; coerência 594 / 3.559 / 278 / 702,
0 falhas; verifica_lancamento 25 / 0.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0146uBo6FVJ2cyEehyP8rK61
</commit_message>
<xml_diff>
--- a/projetos/gestao-ia-planilhas/produto/kit-advogados/19-metas-do-trimestre.xlsx
+++ b/projetos/gestao-ia-planilhas/produto/kit-advogados/19-metas-do-trimestre.xlsx
@@ -1055,7 +1055,7 @@
       </c>
       <c r="F5" s="12" t="n"/>
       <c r="G5" s="18">
-        <f>IFERROR(AVERAGEIFS(Metas!$H$5:$H$13,Metas!$B$5:$B$13,"&lt;&gt;"),0)</f>
+        <f>IF(COUNT(Metas!$H$5:$H$13)=0,"Faltam dados",AVERAGEIFS(Metas!$H$5:$H$13,Metas!$B$5:$B$13,"&lt;&gt;"))</f>
         <v>0.601505376344086</v>
       </c>
       <c r="H5" s="14" t="n"/>
@@ -1111,7 +1111,7 @@
         <v>3</v>
       </c>
       <c r="C9" s="25">
-        <f>IF(OR(Metas!$A$5="",B9=0),"",AVERAGEIFS(Metas!$H$5:$H$7,Metas!$B$5:$B$7,"&lt;&gt;"))</f>
+        <f>IF(OR(Metas!$A$5="",B9=0),"",IF(COUNT(Metas!$H$5:$H$7)=0,"Faltam dados",AVERAGEIFS(Metas!$H$5:$H$7,Metas!$B$5:$B$7,"&lt;&gt;")))</f>
         <v>0.368333333333333</v>
       </c>
       <c r="D9" s="24">
@@ -1123,7 +1123,7 @@
         <v>2</v>
       </c>
       <c r="F9" s="26" t="str">
-        <f>IF(C9="","",REPT("█",ROUND(C9*30,0)))</f>
+        <f>IF(ISNUMBER(C9),REPT("█",ROUND(C9*30,0)),"")</f>
         <v>███████████</v>
       </c>
       <c r="G9" s="21" t="n"/>
@@ -1139,7 +1139,7 @@
         <v>2</v>
       </c>
       <c r="C10" s="25">
-        <f>IF(OR(Metas!$A$8="",B10=0),"",AVERAGEIFS(Metas!$H$8:$H$10,Metas!$B$8:$B$10,"&lt;&gt;"))</f>
+        <f>IF(OR(Metas!$A$8="",B10=0),"",IF(COUNT(Metas!$H$8:$H$10)=0,"Faltam dados",AVERAGEIFS(Metas!$H$8:$H$10,Metas!$B$8:$B$10,"&lt;&gt;")))</f>
         <v>0.786854838709677</v>
       </c>
       <c r="D10" s="24">
@@ -1151,7 +1151,7 @@
         <v>0</v>
       </c>
       <c r="F10" s="26" t="str">
-        <f>IF(C10="","",REPT("█",ROUND(C10*30,0)))</f>
+        <f>IF(ISNUMBER(C10),REPT("█",ROUND(C10*30,0)),"")</f>
         <v>████████████████████████</v>
       </c>
       <c r="G10" s="21" t="n"/>
@@ -1167,7 +1167,7 @@
         <v>3</v>
       </c>
       <c r="C11" s="25">
-        <f>IF(OR(Metas!$A$11="",B11=0),"",AVERAGEIFS(Metas!$H$11:$H$13,Metas!$B$11:$B$13,"&lt;&gt;"))</f>
+        <f>IF(OR(Metas!$A$11="",B11=0),"",IF(COUNT(Metas!$H$11:$H$13)=0,"Faltam dados",AVERAGEIFS(Metas!$H$11:$H$13,Metas!$B$11:$B$13,"&lt;&gt;")))</f>
         <v>0.711111111111111</v>
       </c>
       <c r="D11" s="24">
@@ -1179,7 +1179,7 @@
         <v>1</v>
       </c>
       <c r="F11" s="26" t="str">
-        <f>IF(C11="","",REPT("█",ROUND(C11*30,0)))</f>
+        <f>IF(ISNUMBER(C11),REPT("█",ROUND(C11*30,0)),"")</f>
         <v>█████████████████████</v>
       </c>
       <c r="G11" s="21" t="n"/>
@@ -1901,7 +1901,7 @@
         <v>4.6</v>
       </c>
       <c r="H5" s="25">
-        <f>IF(B5="","",IF(OR(NOT(ISNUMBER(E5)),NOT(ISNUMBER(F5)),NOT(ISNUMBER(G5))),"",IF(K5="Menor é melhor",IF(G5&lt;=F5,1,IF(E5&gt;F5,MAX(0,(E5-G5)/(E5-F5)),MAX(0,1-(G5-F5)/MAX(ABS(F5),ABS(G5))))),IF(G5&gt;=F5,1,IF(E5&lt;F5,MAX(0,(G5-E5)/(F5-E5)),MAX(0,1-(F5-G5)/MAX(ABS(F5),ABS(G5))))))))</f>
+        <f>IF(B5="","",IF(OR(NOT(ISNUMBER(E5)),NOT(ISNUMBER(F5)),NOT(ISNUMBER(G5)),AND(K5&lt;&gt;"Menor é melhor",K5&lt;&gt;"Maior é melhor")),"",IF(K5="Menor é melhor",IF(G5&lt;=F5,1,IF(E5&gt;F5,MAX(0,(E5-G5)/(E5-F5)),MAX(0,1-(G5-F5)/MAX(ABS(F5),ABS(G5))))),IF(G5&gt;=F5,1,IF(E5&lt;F5,MAX(0,(G5-E5)/(F5-E5)),MAX(0,1-(F5-G5)/MAX(ABS(F5),ABS(G5))))))))</f>
         <v>0</v>
       </c>
       <c r="I5" s="25">
@@ -1950,7 +1950,7 @@
         <v>12000</v>
       </c>
       <c r="H6" s="25">
-        <f>IF(B6="","",IF(OR(NOT(ISNUMBER(E6)),NOT(ISNUMBER(F6)),NOT(ISNUMBER(G6))),"",IF(K6="Menor é melhor",IF(G6&lt;=F6,1,IF(E6&gt;F6,MAX(0,(E6-G6)/(E6-F6)),MAX(0,1-(G6-F6)/MAX(ABS(F6),ABS(G6))))),IF(G6&gt;=F6,1,IF(E6&lt;F6,MAX(0,(G6-E6)/(F6-E6)),MAX(0,1-(F6-G6)/MAX(ABS(F6),ABS(G6))))))))</f>
+        <f>IF(B6="","",IF(OR(NOT(ISNUMBER(E6)),NOT(ISNUMBER(F6)),NOT(ISNUMBER(G6)),AND(K6&lt;&gt;"Menor é melhor",K6&lt;&gt;"Maior é melhor")),"",IF(K6="Menor é melhor",IF(G6&lt;=F6,1,IF(E6&gt;F6,MAX(0,(E6-G6)/(E6-F6)),MAX(0,1-(G6-F6)/MAX(ABS(F6),ABS(G6))))),IF(G6&gt;=F6,1,IF(E6&lt;F6,MAX(0,(G6-E6)/(F6-E6)),MAX(0,1-(F6-G6)/MAX(ABS(F6),ABS(G6))))))))</f>
         <v>0.48</v>
       </c>
       <c r="I6" s="25">
@@ -1999,7 +1999,7 @@
         <v>9400</v>
       </c>
       <c r="H7" s="25">
-        <f>IF(B7="","",IF(OR(NOT(ISNUMBER(E7)),NOT(ISNUMBER(F7)),NOT(ISNUMBER(G7))),"",IF(K7="Menor é melhor",IF(G7&lt;=F7,1,IF(E7&gt;F7,MAX(0,(E7-G7)/(E7-F7)),MAX(0,1-(G7-F7)/MAX(ABS(F7),ABS(G7))))),IF(G7&gt;=F7,1,IF(E7&lt;F7,MAX(0,(G7-E7)/(F7-E7)),MAX(0,1-(F7-G7)/MAX(ABS(F7),ABS(G7))))))))</f>
+        <f>IF(B7="","",IF(OR(NOT(ISNUMBER(E7)),NOT(ISNUMBER(F7)),NOT(ISNUMBER(G7)),AND(K7&lt;&gt;"Menor é melhor",K7&lt;&gt;"Maior é melhor")),"",IF(K7="Menor é melhor",IF(G7&lt;=F7,1,IF(E7&gt;F7,MAX(0,(E7-G7)/(E7-F7)),MAX(0,1-(G7-F7)/MAX(ABS(F7),ABS(G7))))),IF(G7&gt;=F7,1,IF(E7&lt;F7,MAX(0,(G7-E7)/(F7-E7)),MAX(0,1-(F7-G7)/MAX(ABS(F7),ABS(G7))))))))</f>
         <v>0.625</v>
       </c>
       <c r="I7" s="25">
@@ -2052,7 +2052,7 @@
         <v>79.5</v>
       </c>
       <c r="H8" s="25">
-        <f>IF(B8="","",IF(OR(NOT(ISNUMBER(E8)),NOT(ISNUMBER(F8)),NOT(ISNUMBER(G8))),"",IF(K8="Menor é melhor",IF(G8&lt;=F8,1,IF(E8&gt;F8,MAX(0,(E8-G8)/(E8-F8)),MAX(0,1-(G8-F8)/MAX(ABS(F8),ABS(G8))))),IF(G8&gt;=F8,1,IF(E8&lt;F8,MAX(0,(G8-E8)/(F8-E8)),MAX(0,1-(F8-G8)/MAX(ABS(F8),ABS(G8))))))))</f>
+        <f>IF(B8="","",IF(OR(NOT(ISNUMBER(E8)),NOT(ISNUMBER(F8)),NOT(ISNUMBER(G8)),AND(K8&lt;&gt;"Menor é melhor",K8&lt;&gt;"Maior é melhor")),"",IF(K8="Menor é melhor",IF(G8&lt;=F8,1,IF(E8&gt;F8,MAX(0,(E8-G8)/(E8-F8)),MAX(0,1-(G8-F8)/MAX(ABS(F8),ABS(G8))))),IF(G8&gt;=F8,1,IF(E8&lt;F8,MAX(0,(G8-E8)/(F8-E8)),MAX(0,1-(F8-G8)/MAX(ABS(F8),ABS(G8))))))))</f>
         <v>0.838709677419355</v>
       </c>
       <c r="I8" s="25">
@@ -2101,7 +2101,7 @@
         <v>514.5</v>
       </c>
       <c r="H9" s="25">
-        <f>IF(B9="","",IF(OR(NOT(ISNUMBER(E9)),NOT(ISNUMBER(F9)),NOT(ISNUMBER(G9))),"",IF(K9="Menor é melhor",IF(G9&lt;=F9,1,IF(E9&gt;F9,MAX(0,(E9-G9)/(E9-F9)),MAX(0,1-(G9-F9)/MAX(ABS(F9),ABS(G9))))),IF(G9&gt;=F9,1,IF(E9&lt;F9,MAX(0,(G9-E9)/(F9-E9)),MAX(0,1-(F9-G9)/MAX(ABS(F9),ABS(G9))))))))</f>
+        <f>IF(B9="","",IF(OR(NOT(ISNUMBER(E9)),NOT(ISNUMBER(F9)),NOT(ISNUMBER(G9)),AND(K9&lt;&gt;"Menor é melhor",K9&lt;&gt;"Maior é melhor")),"",IF(K9="Menor é melhor",IF(G9&lt;=F9,1,IF(E9&gt;F9,MAX(0,(E9-G9)/(E9-F9)),MAX(0,1-(G9-F9)/MAX(ABS(F9),ABS(G9))))),IF(G9&gt;=F9,1,IF(E9&lt;F9,MAX(0,(G9-E9)/(F9-E9)),MAX(0,1-(F9-G9)/MAX(ABS(F9),ABS(G9))))))))</f>
         <v>0.735</v>
       </c>
       <c r="I9" s="25">
@@ -2132,7 +2132,7 @@
       <c r="F10" s="36" t="n"/>
       <c r="G10" s="36" t="n"/>
       <c r="H10" s="25">
-        <f>IF(B10="","",IF(OR(NOT(ISNUMBER(E10)),NOT(ISNUMBER(F10)),NOT(ISNUMBER(G10))),"",IF(K10="Menor é melhor",IF(G10&lt;=F10,1,IF(E10&gt;F10,MAX(0,(E10-G10)/(E10-F10)),MAX(0,1-(G10-F10)/MAX(ABS(F10),ABS(G10))))),IF(G10&gt;=F10,1,IF(E10&lt;F10,MAX(0,(G10-E10)/(F10-E10)),MAX(0,1-(F10-G10)/MAX(ABS(F10),ABS(G10))))))))</f>
+        <f>IF(B10="","",IF(OR(NOT(ISNUMBER(E10)),NOT(ISNUMBER(F10)),NOT(ISNUMBER(G10)),AND(K10&lt;&gt;"Menor é melhor",K10&lt;&gt;"Maior é melhor")),"",IF(K10="Menor é melhor",IF(G10&lt;=F10,1,IF(E10&gt;F10,MAX(0,(E10-G10)/(E10-F10)),MAX(0,1-(G10-F10)/MAX(ABS(F10),ABS(G10))))),IF(G10&gt;=F10,1,IF(E10&lt;F10,MAX(0,(G10-E10)/(F10-E10)),MAX(0,1-(F10-G10)/MAX(ABS(F10),ABS(G10))))))))</f>
         <v/>
       </c>
       <c r="I10" s="25">
@@ -2177,7 +2177,7 @@
         <v>6</v>
       </c>
       <c r="H11" s="25">
-        <f>IF(B11="","",IF(OR(NOT(ISNUMBER(E11)),NOT(ISNUMBER(F11)),NOT(ISNUMBER(G11))),"",IF(K11="Menor é melhor",IF(G11&lt;=F11,1,IF(E11&gt;F11,MAX(0,(E11-G11)/(E11-F11)),MAX(0,1-(G11-F11)/MAX(ABS(F11),ABS(G11))))),IF(G11&gt;=F11,1,IF(E11&lt;F11,MAX(0,(G11-E11)/(F11-E11)),MAX(0,1-(F11-G11)/MAX(ABS(F11),ABS(G11))))))))</f>
+        <f>IF(B11="","",IF(OR(NOT(ISNUMBER(E11)),NOT(ISNUMBER(F11)),NOT(ISNUMBER(G11)),AND(K11&lt;&gt;"Menor é melhor",K11&lt;&gt;"Maior é melhor")),"",IF(K11="Menor é melhor",IF(G11&lt;=F11,1,IF(E11&gt;F11,MAX(0,(E11-G11)/(E11-F11)),MAX(0,1-(G11-F11)/MAX(ABS(F11),ABS(G11))))),IF(G11&gt;=F11,1,IF(E11&lt;F11,MAX(0,(G11-E11)/(F11-E11)),MAX(0,1-(F11-G11)/MAX(ABS(F11),ABS(G11))))))))</f>
         <v>0.75</v>
       </c>
       <c r="I11" s="25">
@@ -2226,7 +2226,7 @@
         <v>53000</v>
       </c>
       <c r="H12" s="25">
-        <f>IF(B12="","",IF(OR(NOT(ISNUMBER(E12)),NOT(ISNUMBER(F12)),NOT(ISNUMBER(G12))),"",IF(K12="Menor é melhor",IF(G12&lt;=F12,1,IF(E12&gt;F12,MAX(0,(E12-G12)/(E12-F12)),MAX(0,1-(G12-F12)/MAX(ABS(F12),ABS(G12))))),IF(G12&gt;=F12,1,IF(E12&lt;F12,MAX(0,(G12-E12)/(F12-E12)),MAX(0,1-(F12-G12)/MAX(ABS(F12),ABS(G12))))))))</f>
+        <f>IF(B12="","",IF(OR(NOT(ISNUMBER(E12)),NOT(ISNUMBER(F12)),NOT(ISNUMBER(G12)),AND(K12&lt;&gt;"Menor é melhor",K12&lt;&gt;"Maior é melhor")),"",IF(K12="Menor é melhor",IF(G12&lt;=F12,1,IF(E12&gt;F12,MAX(0,(E12-G12)/(E12-F12)),MAX(0,1-(G12-F12)/MAX(ABS(F12),ABS(G12))))),IF(G12&gt;=F12,1,IF(E12&lt;F12,MAX(0,(G12-E12)/(F12-E12)),MAX(0,1-(F12-G12)/MAX(ABS(F12),ABS(G12))))))))</f>
         <v>0.883333333333333</v>
       </c>
       <c r="I12" s="25">
@@ -2275,7 +2275,7 @@
         <v>1</v>
       </c>
       <c r="H13" s="25">
-        <f>IF(B13="","",IF(OR(NOT(ISNUMBER(E13)),NOT(ISNUMBER(F13)),NOT(ISNUMBER(G13))),"",IF(K13="Menor é melhor",IF(G13&lt;=F13,1,IF(E13&gt;F13,MAX(0,(E13-G13)/(E13-F13)),MAX(0,1-(G13-F13)/MAX(ABS(F13),ABS(G13))))),IF(G13&gt;=F13,1,IF(E13&lt;F13,MAX(0,(G13-E13)/(F13-E13)),MAX(0,1-(F13-G13)/MAX(ABS(F13),ABS(G13))))))))</f>
+        <f>IF(B13="","",IF(OR(NOT(ISNUMBER(E13)),NOT(ISNUMBER(F13)),NOT(ISNUMBER(G13)),AND(K13&lt;&gt;"Menor é melhor",K13&lt;&gt;"Maior é melhor")),"",IF(K13="Menor é melhor",IF(G13&lt;=F13,1,IF(E13&gt;F13,MAX(0,(E13-G13)/(E13-F13)),MAX(0,1-(G13-F13)/MAX(ABS(F13),ABS(G13))))),IF(G13&gt;=F13,1,IF(E13&lt;F13,MAX(0,(G13-E13)/(F13-E13)),MAX(0,1-(F13-G13)/MAX(ABS(F13),ABS(G13))))))))</f>
         <v>0.5</v>
       </c>
       <c r="I13" s="25">
@@ -2300,7 +2300,7 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Progresso: só é calculado com ponto de partida, meta e valor atual preenchidos (zero vale; vazio vira "Faltam dados" e fica fora das contagens). Valor atual no alvo = 100 %. Fora do alvo, é o caminho andado entre o ponto de partida e a meta; quando o ponto de partida já estava dentro da meta (um limite a manter), é a distância ao limite: para um teto ("Menor é melhor"), meta ÷ atual (16 para um teto de 8 = 50 %); para um piso ("Maior é melhor"), atual ÷ meta (4 para um piso de 8 = 50 %). Com zero ou valores negativos (um limite de prejuízo, por exemplo) a conta usa o maior valor absoluto como escala e nunca dá 100 % sem o alvo estar cumprido. Semáforo: Atingido (100%); No ritmo (progresso até 10 pontos abaixo do tempo decorrido); Atenção (até 25 pontos abaixo); Em risco (mais que isso). A planilha avisa; a ação é do escritório.</t>
+          <t>Progresso: só é calculado com ponto de partida, meta, valor atual e sentido preenchidos (zero vale; vazio vira "Faltam dados" e fica fora das contagens; sem nenhuma medição, a média do Painel também diz "Faltam dados"). Valor atual no alvo = 100 %. Fora do alvo, é o caminho andado entre o ponto de partida e a meta; quando o ponto de partida já estava dentro da meta (um limite a manter), é a distância ao limite: para um teto ("Menor é melhor"), meta ÷ atual (16 para um teto de 8 = 50 %); para um piso ("Maior é melhor"), atual ÷ meta (4 para um piso de 8 = 50 %). Com zero ou valores negativos (um limite de prejuízo, por exemplo) a conta usa o maior valor absoluto como escala e nunca dá 100 % sem o alvo estar cumprido. Semáforo: Atingido (100%); No ritmo (progresso até 10 pontos abaixo do tempo decorrido); Atenção (até 25 pontos abaixo); Em risco (mais que isso). A planilha avisa; a ação é do escritório.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Planilhas: aplicar a rodada 8 da auditoria (metas: espelhos de Atual e Meta sem zero falso)
Um achado nas três planilhas de metas (06 Completo, 19 Advogados, 19 Médicos),
reproduzido antes de corrigir: referência a célula vazia virava 0 nos espelhos de
Atual e Meta (Painel, Semanas) e, no Completo, nos "ganho" e "falta" da aba Meses
(ponto de partida apagado dava ganho de 27.400; meta apagada dava falta de −27.400).

- Espelhos só copiam número (ISNUMBER); ganho e falta de Meses exigem os dois
  operandos numéricos; o IFERROR(...,0) saiu. Zero digitado continua zero.

Travas: recalc_todos 189.771 fórmulas / 0 erro; coerência 594 / 3.559 / 278 / 702,
0 falhas; verifica_lancamento 25 / 0.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0146uBo6FVJ2cyEehyP8rK61
</commit_message>
<xml_diff>
--- a/projetos/gestao-ia-planilhas/produto/kit-advogados/19-metas-do-trimestre.xlsx
+++ b/projetos/gestao-ia-planilhas/produto/kit-advogados/19-metas-do-trimestre.xlsx
@@ -1244,11 +1244,11 @@
         <v>Rafael Lima</v>
       </c>
       <c r="C15" s="28">
-        <f>IF(Metas!B5="","",Metas!G5)</f>
+        <f>IF(OR(Metas!B5="",NOT(ISNUMBER(Metas!G5))),"",Metas!G5)</f>
         <v>4.6</v>
       </c>
       <c r="D15" s="28">
-        <f>IF(Metas!B5="","",Metas!F5)</f>
+        <f>IF(OR(Metas!B5="",NOT(ISNUMBER(Metas!F5))),"",Metas!F5)</f>
         <v>3</v>
       </c>
       <c r="E15" s="25">
@@ -1278,11 +1278,11 @@
         <v>Marina Ferraz</v>
       </c>
       <c r="C16" s="28">
-        <f>IF(Metas!B6="","",Metas!G6)</f>
+        <f>IF(OR(Metas!B6="",NOT(ISNUMBER(Metas!G6))),"",Metas!G6)</f>
         <v>12000</v>
       </c>
       <c r="D16" s="28">
-        <f>IF(Metas!B6="","",Metas!F6)</f>
+        <f>IF(OR(Metas!B6="",NOT(ISNUMBER(Metas!F6))),"",Metas!F6)</f>
         <v>18500</v>
       </c>
       <c r="E16" s="25">
@@ -1312,11 +1312,11 @@
         <v>Marina Ferraz</v>
       </c>
       <c r="C17" s="28">
-        <f>IF(Metas!B7="","",Metas!G7)</f>
+        <f>IF(OR(Metas!B7="",NOT(ISNUMBER(Metas!G7))),"",Metas!G7)</f>
         <v>9400</v>
       </c>
       <c r="D17" s="28">
-        <f>IF(Metas!B7="","",Metas!F7)</f>
+        <f>IF(OR(Metas!B7="",NOT(ISNUMBER(Metas!F7))),"",Metas!F7)</f>
         <v>11320</v>
       </c>
       <c r="E17" s="25">
@@ -1346,11 +1346,11 @@
         <v>Rafael Lima</v>
       </c>
       <c r="C18" s="28">
-        <f>IF(Metas!B8="","",Metas!G8)</f>
+        <f>IF(OR(Metas!B8="",NOT(ISNUMBER(Metas!G8))),"",Metas!G8)</f>
         <v>79.5</v>
       </c>
       <c r="D18" s="28">
-        <f>IF(Metas!B8="","",Metas!F8)</f>
+        <f>IF(OR(Metas!B8="",NOT(ISNUMBER(Metas!F8))),"",Metas!F8)</f>
         <v>80</v>
       </c>
       <c r="E18" s="25">
@@ -1380,11 +1380,11 @@
         <v>Marina Ferraz</v>
       </c>
       <c r="C19" s="28">
-        <f>IF(Metas!B9="","",Metas!G9)</f>
+        <f>IF(OR(Metas!B9="",NOT(ISNUMBER(Metas!G9))),"",Metas!G9)</f>
         <v>514.5</v>
       </c>
       <c r="D19" s="28">
-        <f>IF(Metas!B9="","",Metas!F9)</f>
+        <f>IF(OR(Metas!B9="",NOT(ISNUMBER(Metas!F9))),"",Metas!F9)</f>
         <v>700</v>
       </c>
       <c r="E19" s="25">
@@ -1414,11 +1414,11 @@
         <v/>
       </c>
       <c r="C20" s="28">
-        <f>IF(Metas!B10="","",Metas!G10)</f>
+        <f>IF(OR(Metas!B10="",NOT(ISNUMBER(Metas!G10))),"",Metas!G10)</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>IF(Metas!B10="","",Metas!F10)</f>
+        <f>IF(OR(Metas!B10="",NOT(ISNUMBER(Metas!F10))),"",Metas!F10)</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -1448,11 +1448,11 @@
         <v>Marina Ferraz</v>
       </c>
       <c r="C21" s="28">
-        <f>IF(Metas!B11="","",Metas!G11)</f>
+        <f>IF(OR(Metas!B11="",NOT(ISNUMBER(Metas!G11))),"",Metas!G11)</f>
         <v>6</v>
       </c>
       <c r="D21" s="28">
-        <f>IF(Metas!B11="","",Metas!F11)</f>
+        <f>IF(OR(Metas!B11="",NOT(ISNUMBER(Metas!F11))),"",Metas!F11)</f>
         <v>8</v>
       </c>
       <c r="E21" s="25">
@@ -1482,11 +1482,11 @@
         <v>Marina Ferraz</v>
       </c>
       <c r="C22" s="28">
-        <f>IF(Metas!B12="","",Metas!G12)</f>
+        <f>IF(OR(Metas!B12="",NOT(ISNUMBER(Metas!G12))),"",Metas!G12)</f>
         <v>53000</v>
       </c>
       <c r="D22" s="28">
-        <f>IF(Metas!B12="","",Metas!F12)</f>
+        <f>IF(OR(Metas!B12="",NOT(ISNUMBER(Metas!F12))),"",Metas!F12)</f>
         <v>60000</v>
       </c>
       <c r="E22" s="25">
@@ -1516,11 +1516,11 @@
         <v>Rafael Lima</v>
       </c>
       <c r="C23" s="28">
-        <f>IF(Metas!B13="","",Metas!G13)</f>
+        <f>IF(OR(Metas!B13="",NOT(ISNUMBER(Metas!G13))),"",Metas!G13)</f>
         <v>1</v>
       </c>
       <c r="D23" s="28">
-        <f>IF(Metas!B13="","",Metas!F13)</f>
+        <f>IF(OR(Metas!B13="",NOT(ISNUMBER(Metas!F13))),"",Metas!F13)</f>
         <v>0</v>
       </c>
       <c r="E23" s="25">
@@ -2474,7 +2474,7 @@
         <v>Inadimplência: vencido ÷ (pago + vencido) (%)</v>
       </c>
       <c r="B5" s="24">
-        <f>IF(Metas!B5="","",Metas!F5)</f>
+        <f>IF(OR(Metas!B5="",NOT(ISNUMBER(Metas!F5))),"",Metas!F5)</f>
         <v>3</v>
       </c>
       <c r="C5" s="36" t="n">
@@ -2519,7 +2519,7 @@
         <v>Reserva guardada em conta separada (R$)</v>
       </c>
       <c r="B6" s="24">
-        <f>IF(Metas!B6="","",Metas!F6)</f>
+        <f>IF(OR(Metas!B6="",NOT(ISNUMBER(Metas!F6))),"",Metas!F6)</f>
         <v>18500</v>
       </c>
       <c r="C6" s="36" t="n">
@@ -2564,7 +2564,7 @@
         <v>Conta de provisão de impostos, 13º e férias (R$)</v>
       </c>
       <c r="B7" s="24">
-        <f>IF(Metas!B7="","",Metas!F7)</f>
+        <f>IF(OR(Metas!B7="",NOT(ISNUMBER(Metas!F7))),"",Metas!F7)</f>
         <v>11320</v>
       </c>
       <c r="C7" s="36" t="n">
@@ -2609,7 +2609,7 @@
         <v>Horas faturáveis no mês (%)</v>
       </c>
       <c r="B8" s="24">
-        <f>IF(Metas!B8="","",Metas!F8)</f>
+        <f>IF(OR(Metas!B8="",NOT(ISNUMBER(Metas!F8))),"",Metas!F8)</f>
         <v>80</v>
       </c>
       <c r="C8" s="36" t="n">
@@ -2654,7 +2654,7 @@
         <v>Horas faturáveis lançadas no trimestre (h)</v>
       </c>
       <c r="B9" s="24">
-        <f>IF(Metas!B9="","",Metas!F9)</f>
+        <f>IF(OR(Metas!B9="",NOT(ISNUMBER(Metas!F9))),"",Metas!F9)</f>
         <v>700</v>
       </c>
       <c r="C9" s="36" t="n">
@@ -2699,7 +2699,7 @@
         <v/>
       </c>
       <c r="B10" s="24">
-        <f>IF(Metas!B10="","",Metas!F10)</f>
+        <f>IF(OR(Metas!B10="",NOT(ISNUMBER(Metas!F10))),"",Metas!F10)</f>
         <v/>
       </c>
       <c r="C10" s="36" t="n"/>
@@ -2722,7 +2722,7 @@
         <v>Propostas fechadas no trimestre</v>
       </c>
       <c r="B11" s="24">
-        <f>IF(Metas!B11="","",Metas!F11)</f>
+        <f>IF(OR(Metas!B11="",NOT(ISNUMBER(Metas!F11))),"",Metas!F11)</f>
         <v>8</v>
       </c>
       <c r="C11" s="36" t="n">
@@ -2767,7 +2767,7 @@
         <v>Honorários fechados no trimestre (R$)</v>
       </c>
       <c r="B12" s="24">
-        <f>IF(Metas!B12="","",Metas!F12)</f>
+        <f>IF(OR(Metas!B12="",NOT(ISNUMBER(Metas!F12))),"",Metas!F12)</f>
         <v>60000</v>
       </c>
       <c r="C12" s="36" t="n">
@@ -2812,7 +2812,7 @@
         <v>Propostas paradas há mais de 14 dias</v>
       </c>
       <c r="B13" s="24">
-        <f>IF(Metas!B13="","",Metas!F13)</f>
+        <f>IF(OR(Metas!B13="",NOT(ISNUMBER(Metas!F13))),"",Metas!F13)</f>
         <v>0</v>
       </c>
       <c r="C13" s="36" t="n">

</xml_diff>

<commit_message>
Planilhas: rodada 9 (Dono vazio), inventário dos 53 e prompt da auditoria final
- 06 Completo, 19 Advogados, 19 Médicos: espelho do Dono testa o nome vazio antes de
  copiar (mostrava 0). Único achado da rodada 9, leve.
- inventario.py: abas, fórmulas, entradas, listas, regras condicionais e quatro colunas
  de controle (validação sem bloqueio, célula desbloqueada fora do amarelo, _xlfn,
  regra condicional sem INDIRECT) dos 53 arquivos de entrega; saída em
  auditoria/inventario-2026-09-19.md.
- auditoria/prompt-auditoria-final-2026-09-19.md: pedido da auditoria final completa.
- Triagem com a seção da rodada 9 e o fecho das travas.

Travas: recalc_todos 189.771 fórmulas / 0 erro; coerência 594 / 3.559 / 278 / 702,
0 falhas; verifica_lancamento 25 / 0.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0146uBo6FVJ2cyEehyP8rK61
</commit_message>
<xml_diff>
--- a/projetos/gestao-ia-planilhas/produto/kit-advogados/19-metas-do-trimestre.xlsx
+++ b/projetos/gestao-ia-planilhas/produto/kit-advogados/19-metas-do-trimestre.xlsx
@@ -1240,7 +1240,7 @@
         <v>Inadimplência: vencido ÷ (pago + vencido) (%)</v>
       </c>
       <c r="B15" s="24" t="str">
-        <f>IF(Metas!B5="","",Metas!C5)</f>
+        <f>IF(OR(Metas!B5="",Metas!C5=""),"",Metas!C5)</f>
         <v>Rafael Lima</v>
       </c>
       <c r="C15" s="28">
@@ -1274,7 +1274,7 @@
         <v>Reserva guardada em conta separada (R$)</v>
       </c>
       <c r="B16" s="24" t="str">
-        <f>IF(Metas!B6="","",Metas!C6)</f>
+        <f>IF(OR(Metas!B6="",Metas!C6=""),"",Metas!C6)</f>
         <v>Marina Ferraz</v>
       </c>
       <c r="C16" s="28">
@@ -1308,7 +1308,7 @@
         <v>Conta de provisão de impostos, 13º e férias (R$)</v>
       </c>
       <c r="B17" s="24" t="str">
-        <f>IF(Metas!B7="","",Metas!C7)</f>
+        <f>IF(OR(Metas!B7="",Metas!C7=""),"",Metas!C7)</f>
         <v>Marina Ferraz</v>
       </c>
       <c r="C17" s="28">
@@ -1342,7 +1342,7 @@
         <v>Horas faturáveis no mês (%)</v>
       </c>
       <c r="B18" s="24" t="str">
-        <f>IF(Metas!B8="","",Metas!C8)</f>
+        <f>IF(OR(Metas!B8="",Metas!C8=""),"",Metas!C8)</f>
         <v>Rafael Lima</v>
       </c>
       <c r="C18" s="28">
@@ -1376,7 +1376,7 @@
         <v>Horas faturáveis lançadas no trimestre (h)</v>
       </c>
       <c r="B19" s="24" t="str">
-        <f>IF(Metas!B9="","",Metas!C9)</f>
+        <f>IF(OR(Metas!B9="",Metas!C9=""),"",Metas!C9)</f>
         <v>Marina Ferraz</v>
       </c>
       <c r="C19" s="28">
@@ -1410,7 +1410,7 @@
         <v/>
       </c>
       <c r="B20" s="24">
-        <f>IF(Metas!B10="","",Metas!C10)</f>
+        <f>IF(OR(Metas!B10="",Metas!C10=""),"",Metas!C10)</f>
         <v/>
       </c>
       <c r="C20" s="28">
@@ -1444,7 +1444,7 @@
         <v>Propostas fechadas no trimestre</v>
       </c>
       <c r="B21" s="24" t="str">
-        <f>IF(Metas!B11="","",Metas!C11)</f>
+        <f>IF(OR(Metas!B11="",Metas!C11=""),"",Metas!C11)</f>
         <v>Marina Ferraz</v>
       </c>
       <c r="C21" s="28">
@@ -1478,7 +1478,7 @@
         <v>Honorários fechados no trimestre (R$)</v>
       </c>
       <c r="B22" s="24" t="str">
-        <f>IF(Metas!B12="","",Metas!C12)</f>
+        <f>IF(OR(Metas!B12="",Metas!C12=""),"",Metas!C12)</f>
         <v>Marina Ferraz</v>
       </c>
       <c r="C22" s="28">
@@ -1512,7 +1512,7 @@
         <v>Propostas paradas há mais de 14 dias</v>
       </c>
       <c r="B23" s="24" t="str">
-        <f>IF(Metas!B13="","",Metas!C13)</f>
+        <f>IF(OR(Metas!B13="",Metas!C13=""),"",Metas!C13)</f>
         <v>Rafael Lima</v>
       </c>
       <c r="C23" s="28">

</xml_diff>